<commit_message>
[Add] 2026-05-26 Todo List
</commit_message>
<xml_diff>
--- a/docs/table_column_mapping.xlsx
+++ b/docs/table_column_mapping.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>RequiredHours</t>
+          <t>Hours</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -1622,13 +1622,13 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>建立時帶入，唯讀</t>
+          <t>訓練時數</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="n"/>
-      <c r="B35" s="9" t="n"/>
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="n"/>
       <c r="C35" s="7" t="inlineStr">
         <is>
           <t>TA005</t>
@@ -1657,54 +1657,54 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="9" t="n"/>
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>TA006</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>有效年限</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>TCSTB</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>TrainingDetail (訓練明細)</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>COMPANY</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>COMPANY</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>varchar(10)</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>公司代碼（系統欄位）</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>建立者（系統欄位）</t>
+          <t>公司代碼（系統欄位）</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1729,12 @@
       <c r="B38" s="4" t="n"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>USR_GROUP</t>
+          <t>CREATOR</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>USR_GROUP</t>
+          <t>CREATOR</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>使用者群組（系統欄位）</t>
+          <t>建立者（系統欄位）</t>
         </is>
       </c>
     </row>
@@ -1759,17 +1759,17 @@
       <c r="B39" s="4" t="n"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>CREATE_DATE</t>
+          <t>USR_GROUP</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>CREATE_DATE</t>
+          <t>USR_GROUP</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>char(8)</t>
+          <t>varchar(10)</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>建立日期 YYYYMMDD（系統欄位）</t>
+          <t>使用者群組（系統欄位）</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1789,17 @@
       <c r="B40" s="4" t="n"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>MODIFIER</t>
+          <t>CREATE_DATE</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>MODIFIER</t>
+          <t>CREATE_DATE</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>varchar(10)</t>
+          <t>char(8)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>修改者（系統欄位）</t>
+          <t>建立日期 YYYYMMDD（系統欄位）</t>
         </is>
       </c>
     </row>
@@ -1819,17 +1819,17 @@
       <c r="B41" s="4" t="n"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>MODI_DATE</t>
+          <t>MODIFIER</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>MODI_DATE</t>
+          <t>MODIFIER</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>char(8)</t>
+          <t>varchar(10)</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>修改日期 YYYYMMDD（系統欄位）</t>
+          <t>修改者（系統欄位）</t>
         </is>
       </c>
     </row>
@@ -1849,17 +1849,17 @@
       <c r="B42" s="4" t="n"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>FLAG</t>
+          <t>MODI_DATE</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>FLAG</t>
+          <t>MODI_DATE</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>decimal(3,0)</t>
+          <t>char(8)</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
@@ -1870,41 +1870,37 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>狀態旗標（系統欄位）</t>
+          <t>修改日期 YYYYMMDD（系統欄位）</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
       <c r="B43" s="4" t="n"/>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>TB001</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>EmployeeId</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>varchar(10)</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>PK/FK→TCSTA</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>複合FK→TCSTA cascade delete</t>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>FLAG</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>FLAG</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>decimal(3,0)</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>狀態旗標（系統欄位）</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1909,12 @@
       <c r="B44" s="4" t="n"/>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>TB002</t>
+          <t>TB001</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>LicenseType</t>
+          <t>EmployeeId</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -1947,22 +1943,22 @@
       <c r="B45" s="4" t="n"/>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>TB003</t>
+          <t>TB002</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>TrainingDate</t>
+          <t>LicenseType</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>varchar(10)</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>PK/FK→TCSTA</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -1972,56 +1968,60 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>訓練日期</t>
+          <t>複合FK→TCSTA cascade delete</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
       <c r="B46" s="4" t="n"/>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>TB003</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>TrainingDate</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>訓練日期</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n"/>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>TB004</t>
         </is>
       </c>
-      <c r="D46" s="8" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>TrainingType</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>int</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr"/>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H46" s="8" t="inlineStr">
-        <is>
-          <t>1=取得證照, 2=回訓</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="n"/>
-      <c r="B47" s="9" t="n"/>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>TB005</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Hours</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>decimal(6,1)</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr"/>
@@ -2031,6 +2031,36 @@
         </is>
       </c>
       <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>1=取得證照, 2=回訓</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="n"/>
+      <c r="B48" s="9" t="n"/>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>TB005</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>decimal(6,1)</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
         <is>
           <t>訓練時數</t>
         </is>
@@ -2040,12 +2070,12 @@
   <mergeCells count="8">
     <mergeCell ref="B2:B13"/>
     <mergeCell ref="A2:A13"/>
-    <mergeCell ref="B24:B35"/>
-    <mergeCell ref="A24:A35"/>
-    <mergeCell ref="B36:B47"/>
+    <mergeCell ref="A37:A48"/>
+    <mergeCell ref="A24:A36"/>
     <mergeCell ref="A14:A23"/>
     <mergeCell ref="B14:B23"/>
-    <mergeCell ref="A36:A47"/>
+    <mergeCell ref="B24:B36"/>
+    <mergeCell ref="B37:B48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2813,7 +2843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3159,7 +3189,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>RequiredHours</t>
+          <t>Hours</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -3175,7 +3205,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>建立時帶入，唯讀</t>
+          <t>訓練時數</t>
         </is>
       </c>
     </row>
@@ -3204,6 +3234,34 @@
       <c r="F14" s="8" t="inlineStr">
         <is>
           <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>TA006</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>有效年限</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3668,7 @@
       <c r="D14" s="7" t="inlineStr"/>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">

</xml_diff>